<commit_message>
Rebuild the workbook on the tapered FY2028 base
Sales 3,475.2 GWh, losses 1,291.9, net generation 4,767.1. The generator now
reads FY2026 monthly-by-class from the engine and asserts the tie-out rather
than carrying a pinned figure.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JPS_LE_Sales_Gen_FY2026-28.xlsx
+++ b/JPS_LE_Sales_Gen_FY2026-28.xlsx
@@ -946,43 +946,43 @@
         <v>693810000</v>
       </c>
       <c r="AB7" s="7" t="n">
-        <v>47473607</v>
+        <v>47935473</v>
       </c>
       <c r="AC7" s="7" t="n">
-        <v>44782732</v>
+        <v>45218419</v>
       </c>
       <c r="AD7" s="7" t="n">
-        <v>53130660</v>
+        <v>53647563</v>
       </c>
       <c r="AE7" s="7" t="n">
-        <v>50653862</v>
+        <v>51146668</v>
       </c>
       <c r="AF7" s="7" t="n">
-        <v>59317664</v>
+        <v>59894760</v>
       </c>
       <c r="AG7" s="7" t="n">
-        <v>58955580</v>
+        <v>59529153</v>
       </c>
       <c r="AH7" s="7" t="n">
-        <v>64858838</v>
+        <v>65489843</v>
       </c>
       <c r="AI7" s="7" t="n">
-        <v>65838403</v>
+        <v>66478938</v>
       </c>
       <c r="AJ7" s="7" t="n">
-        <v>63825874</v>
+        <v>64446830</v>
       </c>
       <c r="AK7" s="7" t="n">
-        <v>65839285</v>
+        <v>66479829</v>
       </c>
       <c r="AL7" s="7" t="n">
-        <v>64573575</v>
+        <v>65201804</v>
       </c>
       <c r="AM7" s="7" t="n">
-        <v>63809920</v>
+        <v>64430721</v>
       </c>
       <c r="AN7" s="8" t="n">
-        <v>703060000</v>
+        <v>709900000</v>
       </c>
     </row>
     <row r="8">
@@ -1070,43 +1070,43 @@
         <v>827110000</v>
       </c>
       <c r="AB8" s="7" t="n">
-        <v>59832339</v>
+        <v>60132494</v>
       </c>
       <c r="AC8" s="7" t="n">
-        <v>56425292</v>
+        <v>56708355</v>
       </c>
       <c r="AD8" s="7" t="n">
-        <v>65895050</v>
+        <v>66225620</v>
       </c>
       <c r="AE8" s="7" t="n">
-        <v>63660656</v>
+        <v>63980016</v>
       </c>
       <c r="AF8" s="7" t="n">
-        <v>70406810</v>
+        <v>70760013</v>
       </c>
       <c r="AG8" s="7" t="n">
-        <v>68781729</v>
+        <v>69126780</v>
       </c>
       <c r="AH8" s="7" t="n">
-        <v>74920590</v>
+        <v>75296436</v>
       </c>
       <c r="AI8" s="7" t="n">
-        <v>73093108</v>
+        <v>73459787</v>
       </c>
       <c r="AJ8" s="7" t="n">
-        <v>70253101</v>
+        <v>70605532</v>
       </c>
       <c r="AK8" s="7" t="n">
-        <v>72460508</v>
+        <v>72824014</v>
       </c>
       <c r="AL8" s="7" t="n">
-        <v>71922202</v>
+        <v>72283007</v>
       </c>
       <c r="AM8" s="7" t="n">
-        <v>71628615</v>
+        <v>71987947</v>
       </c>
       <c r="AN8" s="8" t="n">
-        <v>819280000</v>
+        <v>823390000</v>
       </c>
     </row>
     <row r="9">
@@ -1566,43 +1566,43 @@
         <v>3406350000</v>
       </c>
       <c r="AB12" s="9" t="n">
-        <v>245569748</v>
+        <v>246331768</v>
       </c>
       <c r="AC12" s="9" t="n">
-        <v>231516203</v>
+        <v>232234952</v>
       </c>
       <c r="AD12" s="9" t="n">
-        <v>269711939</v>
+        <v>270559411</v>
       </c>
       <c r="AE12" s="9" t="n">
-        <v>261475751</v>
+        <v>262287917</v>
       </c>
       <c r="AF12" s="9" t="n">
-        <v>293049060</v>
+        <v>293979359</v>
       </c>
       <c r="AG12" s="9" t="n">
-        <v>291102858</v>
+        <v>292021482</v>
       </c>
       <c r="AH12" s="9" t="n">
-        <v>317938347</v>
+        <v>318945199</v>
       </c>
       <c r="AI12" s="9" t="n">
-        <v>315239768</v>
+        <v>316246982</v>
       </c>
       <c r="AJ12" s="9" t="n">
-        <v>305743478</v>
+        <v>306716866</v>
       </c>
       <c r="AK12" s="9" t="n">
-        <v>314776125</v>
+        <v>315780174</v>
       </c>
       <c r="AL12" s="9" t="n">
-        <v>310264185</v>
+        <v>311253220</v>
       </c>
       <c r="AM12" s="9" t="n">
-        <v>307902539</v>
+        <v>308882671</v>
       </c>
       <c r="AN12" s="8" t="n">
-        <v>3464290000</v>
+        <v>3475240000</v>
       </c>
     </row>
     <row r="13">
@@ -1711,7 +1711,7 @@
         <v>0.25364529</v>
       </c>
       <c r="AK13" s="10" t="n">
-        <v>0.29109529</v>
+        <v>0.2910952900000001</v>
       </c>
       <c r="AL13" s="10" t="n">
         <v>0.22869529</v>
@@ -1763,40 +1763,40 @@
         <v>0.2710000033313201</v>
       </c>
       <c r="AB14" s="10" t="n">
-        <v>0.2710084242800463</v>
+        <v>0.2710099090349518</v>
       </c>
       <c r="AC14" s="10" t="n">
-        <v>0.2709601743227563</v>
+        <v>0.2709531031715005</v>
       </c>
       <c r="AD14" s="10" t="n">
-        <v>0.2709908497122918</v>
+        <v>0.2709894891292186</v>
       </c>
       <c r="AE14" s="10" t="n">
-        <v>0.2709946504793775</v>
+        <v>0.2709939796164094</v>
       </c>
       <c r="AF14" s="10" t="n">
-        <v>0.2710487959717811</v>
+        <v>0.2710583843781971</v>
       </c>
       <c r="AG14" s="10" t="n">
-        <v>0.2710408190790013</v>
+        <v>0.2710488519537005</v>
       </c>
       <c r="AH14" s="10" t="n">
-        <v>0.2710256565258747</v>
+        <v>0.2710307056762512</v>
       </c>
       <c r="AI14" s="10" t="n">
-        <v>0.271056347072729</v>
+        <v>0.271067131855498</v>
       </c>
       <c r="AJ14" s="10" t="n">
-        <v>0.2710313448514513</v>
+        <v>0.2710373804554943</v>
       </c>
       <c r="AK14" s="10" t="n">
-        <v>0.271062819860822</v>
+        <v>0.2710747437432402</v>
       </c>
       <c r="AL14" s="10" t="n">
-        <v>0.2710028897205262</v>
+        <v>0.2710035495629999</v>
       </c>
       <c r="AM14" s="10" t="n">
-        <v>0.2709999984227078</v>
+        <v>0.2710001015608322</v>
       </c>
     </row>
     <row r="15">
@@ -1884,43 +1884,43 @@
         <v>4672633766</v>
       </c>
       <c r="AB15" s="7" t="n">
-        <v>339933758</v>
+        <v>340988597</v>
       </c>
       <c r="AC15" s="7" t="n">
-        <v>299831367</v>
+        <v>300762204</v>
       </c>
       <c r="AD15" s="7" t="n">
-        <v>381674295</v>
+        <v>382873569</v>
       </c>
       <c r="AE15" s="7" t="n">
-        <v>360107499</v>
+        <v>361226024</v>
       </c>
       <c r="AF15" s="7" t="n">
-        <v>422989417</v>
+        <v>424332217</v>
       </c>
       <c r="AG15" s="7" t="n">
-        <v>396163571</v>
+        <v>397413731</v>
       </c>
       <c r="AH15" s="7" t="n">
-        <v>430021399</v>
+        <v>431383197</v>
       </c>
       <c r="AI15" s="7" t="n">
-        <v>444247006</v>
+        <v>445666408</v>
       </c>
       <c r="AJ15" s="7" t="n">
-        <v>409649024</v>
+        <v>410953212</v>
       </c>
       <c r="AK15" s="7" t="n">
-        <v>444031645</v>
+        <v>445447984</v>
       </c>
       <c r="AL15" s="7" t="n">
-        <v>402258901</v>
+        <v>403541189</v>
       </c>
       <c r="AM15" s="7" t="n">
-        <v>421204589</v>
+        <v>422545391</v>
       </c>
       <c r="AN15" s="8" t="n">
-        <v>4752112473</v>
+        <v>4767133723</v>
       </c>
     </row>
   </sheetData>

</xml_diff>